<commit_message>
fix the datapoint in MOF-808 and redraw
</commit_message>
<xml_diff>
--- a/external_test/extend-data.xlsx
+++ b/external_test/extend-data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\642\MOL surface modification\paper\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yibinjiang\Documents\GitHub\mol_acid_modification\external_test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDE1C5EA-8858-4EBE-B3D8-0CF7659F2E35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6760E9F-C4CA-446D-BD05-21327A33F086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TPY-MOL" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,6 @@
     <sheet name="BTB-MOL(THF)" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -93,17 +92,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -136,7 +135,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -415,16 +414,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F51"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="14.625" customWidth="1"/>
-    <col min="4" max="4" width="12.75" customWidth="1"/>
-    <col min="5" max="5" width="9.625" customWidth="1"/>
-    <col min="6" max="6" width="8.5" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -444,7 +443,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -464,7 +463,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -484,7 +483,7 @@
         <v>0.57999999999999996</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -504,7 +503,7 @@
         <v>0.68</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -524,7 +523,7 @@
         <v>0.76</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -544,7 +543,7 @@
         <v>1.42</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -564,7 +563,7 @@
         <v>0.78</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -584,7 +583,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -604,7 +603,7 @@
         <v>1.22</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -624,7 +623,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -644,7 +643,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -664,7 +663,7 @@
         <v>1.36</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -684,7 +683,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -704,7 +703,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -724,7 +723,7 @@
         <v>2.42</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6">
       <c r="A16" t="s">
         <v>10</v>
       </c>
@@ -744,7 +743,7 @@
         <v>2.78</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6">
       <c r="A17" t="s">
         <v>10</v>
       </c>
@@ -764,7 +763,7 @@
         <v>1.02</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6">
       <c r="A18" t="s">
         <v>10</v>
       </c>
@@ -784,7 +783,7 @@
         <v>1.84</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6">
       <c r="A19" t="s">
         <v>10</v>
       </c>
@@ -804,7 +803,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6">
       <c r="A20" t="s">
         <v>10</v>
       </c>
@@ -824,7 +823,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6">
       <c r="A21" t="s">
         <v>10</v>
       </c>
@@ -844,7 +843,7 @@
         <v>3.2</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6">
       <c r="A22" t="s">
         <v>12</v>
       </c>
@@ -864,7 +863,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6">
       <c r="A23" t="s">
         <v>12</v>
       </c>
@@ -884,7 +883,7 @@
         <v>0.32</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6">
       <c r="A24" t="s">
         <v>12</v>
       </c>
@@ -904,7 +903,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -924,7 +923,7 @@
         <v>0.72</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6">
       <c r="A26" t="s">
         <v>12</v>
       </c>
@@ -944,7 +943,7 @@
         <v>1.22</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6">
       <c r="A27" t="s">
         <v>12</v>
       </c>
@@ -964,7 +963,7 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6">
       <c r="A28" t="s">
         <v>12</v>
       </c>
@@ -984,7 +983,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6">
       <c r="A29" t="s">
         <v>12</v>
       </c>
@@ -1004,7 +1003,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6">
       <c r="A30" t="s">
         <v>12</v>
       </c>
@@ -1024,7 +1023,7 @@
         <v>0.76</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6">
       <c r="A31" t="s">
         <v>12</v>
       </c>
@@ -1044,7 +1043,7 @@
         <v>1.56</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6">
       <c r="A32" t="s">
         <v>14</v>
       </c>
@@ -1064,7 +1063,7 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6">
       <c r="A33" t="s">
         <v>14</v>
       </c>
@@ -1084,7 +1083,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6">
       <c r="A34" t="s">
         <v>14</v>
       </c>
@@ -1104,7 +1103,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6">
       <c r="A35" t="s">
         <v>14</v>
       </c>
@@ -1124,7 +1123,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6">
       <c r="A36" t="s">
         <v>14</v>
       </c>
@@ -1144,7 +1143,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6">
       <c r="A37" t="s">
         <v>14</v>
       </c>
@@ -1164,7 +1163,7 @@
         <v>2.2999999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6">
       <c r="A38" t="s">
         <v>14</v>
       </c>
@@ -1184,7 +1183,7 @@
         <v>2.88</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6">
       <c r="A39" t="s">
         <v>14</v>
       </c>
@@ -1204,7 +1203,7 @@
         <v>3.02</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6">
       <c r="A40" t="s">
         <v>14</v>
       </c>
@@ -1224,7 +1223,7 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6">
       <c r="A41" t="s">
         <v>14</v>
       </c>
@@ -1244,7 +1243,7 @@
         <v>3.48</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6">
       <c r="A42" t="s">
         <v>16</v>
       </c>
@@ -1264,7 +1263,7 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6">
       <c r="A43" t="s">
         <v>16</v>
       </c>
@@ -1284,7 +1283,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6">
       <c r="A44" t="s">
         <v>16</v>
       </c>
@@ -1304,7 +1303,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6">
       <c r="A45" t="s">
         <v>16</v>
       </c>
@@ -1324,7 +1323,7 @@
         <v>0.57999999999999996</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6">
       <c r="A46" t="s">
         <v>16</v>
       </c>
@@ -1344,7 +1343,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6">
       <c r="A47" t="s">
         <v>16</v>
       </c>
@@ -1364,7 +1363,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6">
       <c r="A48" t="s">
         <v>16</v>
       </c>
@@ -1384,7 +1383,7 @@
         <v>1.46</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6">
       <c r="A49" t="s">
         <v>16</v>
       </c>
@@ -1404,7 +1403,7 @@
         <v>1.68</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6">
       <c r="A50" t="s">
         <v>16</v>
       </c>
@@ -1424,7 +1423,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6">
       <c r="A51" t="s">
         <v>16</v>
       </c>
@@ -1454,16 +1453,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3695A2D6-F2E0-45B5-B0B5-21DDB6BDB207}">
   <dimension ref="A1:F51"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="11.375" customWidth="1"/>
-    <col min="3" max="3" width="14.625" customWidth="1"/>
-    <col min="4" max="4" width="12.375" customWidth="1"/>
-    <col min="5" max="5" width="9.75" customWidth="1"/>
-    <col min="6" max="6" width="9.25" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" customWidth="1"/>
+    <col min="6" max="6" width="9.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1483,7 +1482,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1503,7 +1502,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1523,7 +1522,7 @@
         <v>0.54</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1543,7 +1542,7 @@
         <v>0.62</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1563,7 +1562,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1583,7 +1582,7 @@
         <v>1.56</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1603,7 +1602,7 @@
         <v>0.74</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1623,7 +1622,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1643,7 +1642,7 @@
         <v>1.24</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1663,7 +1662,7 @@
         <v>1.36</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -1683,7 +1682,7 @@
         <v>1.92</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1703,7 +1702,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -1723,7 +1722,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -1743,7 +1742,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -1763,7 +1762,7 @@
         <v>2.88</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6">
       <c r="A16" t="s">
         <v>10</v>
       </c>
@@ -1783,7 +1782,7 @@
         <v>3.32</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6">
       <c r="A17" t="s">
         <v>10</v>
       </c>
@@ -1803,7 +1802,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6">
       <c r="A18" t="s">
         <v>10</v>
       </c>
@@ -1823,7 +1822,7 @@
         <v>1.94</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6">
       <c r="A19" t="s">
         <v>10</v>
       </c>
@@ -1843,7 +1842,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6">
       <c r="A20" t="s">
         <v>10</v>
       </c>
@@ -1863,7 +1862,7 @@
         <v>2.7</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6">
       <c r="A21" t="s">
         <v>10</v>
       </c>
@@ -1883,7 +1882,7 @@
         <v>3.48</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6">
       <c r="A22" t="s">
         <v>12</v>
       </c>
@@ -1903,7 +1902,7 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6">
       <c r="A23" t="s">
         <v>12</v>
       </c>
@@ -1923,7 +1922,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6">
       <c r="A24" t="s">
         <v>12</v>
       </c>
@@ -1943,7 +1942,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -1963,7 +1962,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6">
       <c r="A26" t="s">
         <v>12</v>
       </c>
@@ -1983,7 +1982,7 @@
         <v>1.4</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6">
       <c r="A27" t="s">
         <v>12</v>
       </c>
@@ -2003,7 +2002,7 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6">
       <c r="A28" t="s">
         <v>12</v>
       </c>
@@ -2023,7 +2022,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6">
       <c r="A29" t="s">
         <v>12</v>
       </c>
@@ -2043,7 +2042,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6">
       <c r="A30" t="s">
         <v>12</v>
       </c>
@@ -2063,7 +2062,7 @@
         <v>0.66</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6">
       <c r="A31" t="s">
         <v>12</v>
       </c>
@@ -2083,7 +2082,7 @@
         <v>1.36</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6">
       <c r="A32" t="s">
         <v>14</v>
       </c>
@@ -2103,7 +2102,7 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6">
       <c r="A33" t="s">
         <v>14</v>
       </c>
@@ -2123,7 +2122,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6">
       <c r="A34" t="s">
         <v>14</v>
       </c>
@@ -2143,7 +2142,7 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6">
       <c r="A35" t="s">
         <v>14</v>
       </c>
@@ -2163,7 +2162,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6">
       <c r="A36" t="s">
         <v>14</v>
       </c>
@@ -2183,7 +2182,7 @@
         <v>0.72</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6">
       <c r="A37" t="s">
         <v>14</v>
       </c>
@@ -2203,7 +2202,7 @@
         <v>2.42</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6">
       <c r="A38" t="s">
         <v>14</v>
       </c>
@@ -2223,7 +2222,7 @@
         <v>2.92</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6">
       <c r="A39" t="s">
         <v>14</v>
       </c>
@@ -2243,7 +2242,7 @@
         <v>3.02</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6">
       <c r="A40" t="s">
         <v>14</v>
       </c>
@@ -2263,7 +2262,7 @@
         <v>3.16</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6">
       <c r="A41" t="s">
         <v>14</v>
       </c>
@@ -2283,7 +2282,7 @@
         <v>3.2</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6">
       <c r="A42" t="s">
         <v>16</v>
       </c>
@@ -2303,7 +2302,7 @@
         <v>0.32</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6">
       <c r="A43" t="s">
         <v>16</v>
       </c>
@@ -2323,7 +2322,7 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6">
       <c r="A44" t="s">
         <v>16</v>
       </c>
@@ -2343,7 +2342,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6">
       <c r="A45" t="s">
         <v>16</v>
       </c>
@@ -2363,7 +2362,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6">
       <c r="A46" t="s">
         <v>16</v>
       </c>
@@ -2383,7 +2382,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6">
       <c r="A47" t="s">
         <v>16</v>
       </c>
@@ -2403,7 +2402,7 @@
         <v>0.94</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6">
       <c r="A48" t="s">
         <v>16</v>
       </c>
@@ -2423,7 +2422,7 @@
         <v>1.4</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6">
       <c r="A49" t="s">
         <v>16</v>
       </c>
@@ -2443,7 +2442,7 @@
         <v>1.68</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6">
       <c r="A50" t="s">
         <v>16</v>
       </c>
@@ -2463,7 +2462,7 @@
         <v>1.86</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6">
       <c r="A51" t="s">
         <v>16</v>
       </c>
@@ -2492,16 +2491,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01F31A51-8624-4769-B4F1-0D72003D4BAF}">
   <dimension ref="A1:F51"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="11.375" customWidth="1"/>
-    <col min="3" max="3" width="13.875" customWidth="1"/>
-    <col min="4" max="4" width="13.25" customWidth="1"/>
-    <col min="5" max="5" width="9.375" customWidth="1"/>
-    <col min="6" max="6" width="8.5" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2521,7 +2520,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -2541,7 +2540,7 @@
         <v>1.02</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2561,7 +2560,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2581,7 +2580,7 @@
         <v>1.86</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2601,7 +2600,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2621,7 +2620,7 @@
         <v>2.86</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -2641,7 +2640,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -2661,7 +2660,7 @@
         <v>3.52</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -2681,7 +2680,7 @@
         <v>4.1399999999999997</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -2701,7 +2700,7 @@
         <v>4.62</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -2721,7 +2720,7 @@
         <v>5.26</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -2741,7 +2740,7 @@
         <v>1.34</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -2761,7 +2760,7 @@
         <v>2.08</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -2781,7 +2780,7 @@
         <v>2.48</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -2801,7 +2800,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6">
       <c r="A16" t="s">
         <v>9</v>
       </c>
@@ -2821,7 +2820,7 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6">
       <c r="A17" t="s">
         <v>9</v>
       </c>
@@ -2841,7 +2840,7 @@
         <v>1.6</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6">
       <c r="A18" t="s">
         <v>9</v>
       </c>
@@ -2861,7 +2860,7 @@
         <v>2.92</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6">
       <c r="A19" t="s">
         <v>9</v>
       </c>
@@ -2881,7 +2880,7 @@
         <v>3.56</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6">
       <c r="A20" t="s">
         <v>9</v>
       </c>
@@ -2901,7 +2900,7 @@
         <v>4.04</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -2921,7 +2920,7 @@
         <v>5.48</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6">
       <c r="A22" t="s">
         <v>11</v>
       </c>
@@ -2941,7 +2940,7 @@
         <v>0.32</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6">
       <c r="A23" t="s">
         <v>11</v>
       </c>
@@ -2961,7 +2960,7 @@
         <v>0.54</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6">
       <c r="A24" t="s">
         <v>11</v>
       </c>
@@ -2981,7 +2980,7 @@
         <v>0.62</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6">
       <c r="A25" t="s">
         <v>11</v>
       </c>
@@ -3001,7 +3000,7 @@
         <v>0.92</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6">
       <c r="A26" t="s">
         <v>11</v>
       </c>
@@ -3021,7 +3020,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6">
       <c r="A27" t="s">
         <v>11</v>
       </c>
@@ -3041,7 +3040,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6">
       <c r="A28" t="s">
         <v>11</v>
       </c>
@@ -3061,7 +3060,7 @@
         <v>1.1599999999999999</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6">
       <c r="A29" t="s">
         <v>11</v>
       </c>
@@ -3081,7 +3080,7 @@
         <v>1.36</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6">
       <c r="A30" t="s">
         <v>11</v>
       </c>
@@ -3101,7 +3100,7 @@
         <v>1.66</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6">
       <c r="A31" t="s">
         <v>11</v>
       </c>
@@ -3121,7 +3120,7 @@
         <v>2.2999999999999998</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6">
       <c r="A32" t="s">
         <v>13</v>
       </c>
@@ -3141,7 +3140,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6">
       <c r="A33" t="s">
         <v>13</v>
       </c>
@@ -3161,7 +3160,7 @@
         <v>1.62</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6">
       <c r="A34" t="s">
         <v>13</v>
       </c>
@@ -3181,7 +3180,7 @@
         <v>1.88</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6">
       <c r="A35" t="s">
         <v>13</v>
       </c>
@@ -3201,7 +3200,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6">
       <c r="A36" t="s">
         <v>13</v>
       </c>
@@ -3221,7 +3220,7 @@
         <v>2.98</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6">
       <c r="A37" t="s">
         <v>13</v>
       </c>
@@ -3241,7 +3240,7 @@
         <v>4.88</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6">
       <c r="A38" t="s">
         <v>13</v>
       </c>
@@ -3261,7 +3260,7 @@
         <v>5.42</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6">
       <c r="A39" t="s">
         <v>13</v>
       </c>
@@ -3281,7 +3280,7 @@
         <v>5.56</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6">
       <c r="A40" t="s">
         <v>13</v>
       </c>
@@ -3297,11 +3296,11 @@
       <c r="E40">
         <v>0.12</v>
       </c>
-      <c r="F40" s="1">
-        <v>2.86</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F40">
+        <v>5.72</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
       <c r="A41" t="s">
         <v>13</v>
       </c>
@@ -3321,7 +3320,7 @@
         <v>5.9</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6">
       <c r="A42" t="s">
         <v>15</v>
       </c>
@@ -3341,7 +3340,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6">
       <c r="A43" t="s">
         <v>15</v>
       </c>
@@ -3361,7 +3360,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6">
       <c r="A44" t="s">
         <v>15</v>
       </c>
@@ -3381,7 +3380,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6">
       <c r="A45" t="s">
         <v>15</v>
       </c>
@@ -3401,7 +3400,7 @@
         <v>2.56</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6">
       <c r="A46" t="s">
         <v>15</v>
       </c>
@@ -3421,7 +3420,7 @@
         <v>3.14</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6">
       <c r="A47" t="s">
         <v>15</v>
       </c>
@@ -3441,7 +3440,7 @@
         <v>3.66</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6">
       <c r="A48" t="s">
         <v>15</v>
       </c>
@@ -3461,7 +3460,7 @@
         <v>4.3</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6">
       <c r="A49" t="s">
         <v>15</v>
       </c>
@@ -3481,7 +3480,7 @@
         <v>4.74</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6">
       <c r="A50" t="s">
         <v>15</v>
       </c>
@@ -3501,7 +3500,7 @@
         <v>4.96</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6">
       <c r="A51" t="s">
         <v>15</v>
       </c>
@@ -3530,16 +3529,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AA89F28-0DB5-4B62-B0E6-13A9A3693465}">
   <dimension ref="A1:F51"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="11.125" customWidth="1"/>
-    <col min="3" max="3" width="14.75" customWidth="1"/>
-    <col min="4" max="4" width="12.625" customWidth="1"/>
-    <col min="5" max="5" width="8.875" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" customWidth="1"/>
+    <col min="5" max="5" width="8.85546875" customWidth="1"/>
     <col min="6" max="6" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3559,7 +3558,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -3579,7 +3578,7 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -3599,7 +3598,7 @@
         <v>0.54</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -3619,7 +3618,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -3639,7 +3638,7 @@
         <v>1.01</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -3659,7 +3658,7 @@
         <v>2.33</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -3679,7 +3678,7 @@
         <v>1.95</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -3699,7 +3698,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -3719,7 +3718,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -3739,7 +3738,7 @@
         <v>3.02</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -3759,7 +3758,7 @@
         <v>3.62</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -3779,7 +3778,7 @@
         <v>2.06</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -3799,7 +3798,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -3819,7 +3818,7 @@
         <v>3.68</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -3839,7 +3838,7 @@
         <v>4.34</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6">
       <c r="A16" t="s">
         <v>10</v>
       </c>
@@ -3859,7 +3858,7 @@
         <v>5.15</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6">
       <c r="A17" t="s">
         <v>10</v>
       </c>
@@ -3879,7 +3878,7 @@
         <v>1.67</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6">
       <c r="A18" t="s">
         <v>10</v>
       </c>
@@ -3899,7 +3898,7 @@
         <v>3.0830000000000002</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6">
       <c r="A19" t="s">
         <v>10</v>
       </c>
@@ -3919,7 +3918,7 @@
         <v>3.19</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6">
       <c r="A20" t="s">
         <v>10</v>
       </c>
@@ -3939,7 +3938,7 @@
         <v>3.87</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6">
       <c r="A21" t="s">
         <v>10</v>
       </c>
@@ -3959,7 +3958,7 @@
         <v>4.37</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6">
       <c r="A22" t="s">
         <v>12</v>
       </c>
@@ -3979,7 +3978,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6">
       <c r="A23" t="s">
         <v>12</v>
       </c>
@@ -3999,7 +3998,7 @@
         <v>0.43</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6">
       <c r="A24" t="s">
         <v>12</v>
       </c>
@@ -4019,7 +4018,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -4039,7 +4038,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6">
       <c r="A26" t="s">
         <v>12</v>
       </c>
@@ -4059,7 +4058,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6">
       <c r="A27" t="s">
         <v>12</v>
       </c>
@@ -4079,7 +4078,7 @@
         <v>0.61</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6">
       <c r="A28" t="s">
         <v>12</v>
       </c>
@@ -4099,7 +4098,7 @@
         <v>1.04</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6">
       <c r="A29" t="s">
         <v>12</v>
       </c>
@@ -4119,7 +4118,7 @@
         <v>1.1299999999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6">
       <c r="A30" t="s">
         <v>12</v>
       </c>
@@ -4139,7 +4138,7 @@
         <v>1.4</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6">
       <c r="A31" t="s">
         <v>12</v>
       </c>
@@ -4159,7 +4158,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6">
       <c r="A32" t="s">
         <v>14</v>
       </c>
@@ -4179,7 +4178,7 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6">
       <c r="A33" t="s">
         <v>14</v>
       </c>
@@ -4199,7 +4198,7 @@
         <v>0.43</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6">
       <c r="A34" t="s">
         <v>14</v>
       </c>
@@ -4219,7 +4218,7 @@
         <v>0.56999999999999995</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6">
       <c r="A35" t="s">
         <v>14</v>
       </c>
@@ -4239,7 +4238,7 @@
         <v>0.66</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6">
       <c r="A36" t="s">
         <v>14</v>
       </c>
@@ -4259,7 +4258,7 @@
         <v>1.1499999999999999</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6">
       <c r="A37" t="s">
         <v>14</v>
       </c>
@@ -4279,7 +4278,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6">
       <c r="A38" t="s">
         <v>14</v>
       </c>
@@ -4299,7 +4298,7 @@
         <v>2.64</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6">
       <c r="A39" t="s">
         <v>14</v>
       </c>
@@ -4319,7 +4318,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6">
       <c r="A40" t="s">
         <v>14</v>
       </c>
@@ -4339,7 +4338,7 @@
         <v>2.88</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6">
       <c r="A41" t="s">
         <v>14</v>
       </c>
@@ -4359,7 +4358,7 @@
         <v>3.13</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6">
       <c r="A42" t="s">
         <v>16</v>
       </c>
@@ -4379,7 +4378,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6">
       <c r="A43" t="s">
         <v>16</v>
       </c>
@@ -4399,7 +4398,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6">
       <c r="A44" t="s">
         <v>16</v>
       </c>
@@ -4419,7 +4418,7 @@
         <v>0.74</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6">
       <c r="A45" t="s">
         <v>16</v>
       </c>
@@ -4439,7 +4438,7 @@
         <v>0.92</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6">
       <c r="A46" t="s">
         <v>16</v>
       </c>
@@ -4459,7 +4458,7 @@
         <v>1.73</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6">
       <c r="A47" t="s">
         <v>16</v>
       </c>
@@ -4479,7 +4478,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6">
       <c r="A48" t="s">
         <v>16</v>
       </c>
@@ -4499,7 +4498,7 @@
         <v>2.08</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6">
       <c r="A49" t="s">
         <v>16</v>
       </c>
@@ -4519,7 +4518,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6">
       <c r="A50" t="s">
         <v>16</v>
       </c>
@@ -4539,7 +4538,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6">
       <c r="A51" t="s">
         <v>16</v>
       </c>
@@ -4568,16 +4567,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AE83F43-87AC-4EC8-8D07-60457BE9DB19}">
   <dimension ref="A1:F11"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="13.125" customWidth="1"/>
-    <col min="3" max="3" width="14.625" customWidth="1"/>
-    <col min="4" max="4" width="13.125" customWidth="1"/>
-    <col min="5" max="5" width="10.25" customWidth="1"/>
-    <col min="6" max="6" width="8.875" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" customWidth="1"/>
+    <col min="5" max="5" width="10.28515625" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4597,7 +4596,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -4617,7 +4616,7 @@
         <v>0.94</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -4637,7 +4636,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -4657,7 +4656,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -4677,7 +4676,7 @@
         <v>1.66</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -4697,7 +4696,7 @@
         <v>1.94</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -4717,7 +4716,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -4737,7 +4736,7 @@
         <v>1.06</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -4757,7 +4756,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -4777,7 +4776,7 @@
         <v>1.46</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -4806,16 +4805,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3385F73C-95E1-4450-B69C-9DFAB5F40DB1}">
   <dimension ref="A1:F11"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="11.75" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="13.25" customWidth="1"/>
-    <col min="5" max="5" width="9.625" customWidth="1"/>
-    <col min="6" max="6" width="9.5" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" customWidth="1"/>
+    <col min="6" max="6" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4835,7 +4834,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -4855,7 +4854,7 @@
         <v>0.74</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -4875,7 +4874,7 @@
         <v>1.06</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -4895,7 +4894,7 @@
         <v>1.1599999999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -4915,7 +4914,7 @@
         <v>1.36</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -4935,7 +4934,7 @@
         <v>1.94</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -4955,7 +4954,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -4975,7 +4974,7 @@
         <v>1.22</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -4995,7 +4994,7 @@
         <v>1.42</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -5015,7 +5014,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>8</v>
       </c>

</xml_diff>